<commit_message>
severity, detection, rpn,d-p gap check
</commit_message>
<xml_diff>
--- a/pfmea_audited.xlsx
+++ b/pfmea_audited.xlsx
@@ -50,7 +50,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="36">
+  <fonts count="37">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
@@ -273,10 +273,16 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00CC0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00CC0000"/>
     </font>
   </fonts>
   <fills count="17">
@@ -683,7 +689,9 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -692,9 +700,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -767,7 +773,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1028,6 +1034,90 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -1036,22 +1126,10 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
@@ -1064,70 +1142,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1167,6 +1181,24 @@
     <xf numFmtId="0" fontId="18" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1176,24 +1208,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="6" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1231,13 +1245,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
@@ -1268,7 +1298,21 @@
     <cellStyle name="Normal 3" xfId="5"/>
     <cellStyle name="Hyperlink 2" xfId="6"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor indexed="10"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor indexed="10"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1431,9 +1475,9 @@
     </from>
     <to>
       <col>17</col>
-      <colOff>323191</colOff>
+      <colOff>327001</colOff>
       <row>2</row>
-      <rowOff>136466</rowOff>
+      <rowOff>132656</rowOff>
     </to>
     <pic>
       <nvPicPr>
@@ -1474,7 +1518,7 @@
     </from>
     <to>
       <col>12</col>
-      <colOff>973276</colOff>
+      <colOff>969466</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </to>
@@ -2210,7 +2254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:X23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.2"/>
   <cols>
     <col width="16.6640625" customWidth="1" min="1" max="1"/>
@@ -2232,7 +2276,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.6" customHeight="1">
-      <c r="A1" s="94" t="inlineStr">
+      <c r="A1" s="91" t="inlineStr">
         <is>
           <t>Quality Tools</t>
         </is>
@@ -2251,13 +2295,13 @@
       <c r="K1" s="19" t="n"/>
       <c r="L1" s="19" t="n"/>
       <c r="O1" s="18" t="n"/>
-      <c r="Q1" s="19" t="n"/>
       <c r="R1" s="19" t="n"/>
-      <c r="S1" s="18" t="n"/>
+      <c r="S1" s="19" t="n"/>
       <c r="T1" s="18" t="n"/>
       <c r="U1" s="18" t="n"/>
       <c r="V1" s="18" t="n"/>
       <c r="W1" s="18" t="n"/>
+      <c r="X1" s="18" t="n"/>
     </row>
     <row r="2" ht="16.2" customHeight="1">
       <c r="A2" s="20" t="inlineStr">
@@ -2275,13 +2319,13 @@
       <c r="K2" s="19" t="n"/>
       <c r="L2" s="19" t="n"/>
       <c r="O2" s="18" t="n"/>
-      <c r="Q2" s="19" t="n"/>
       <c r="R2" s="19" t="n"/>
-      <c r="S2" s="18" t="n"/>
+      <c r="S2" s="19" t="n"/>
       <c r="T2" s="18" t="n"/>
       <c r="U2" s="18" t="n"/>
       <c r="V2" s="18" t="n"/>
       <c r="W2" s="18" t="n"/>
+      <c r="X2" s="18" t="n"/>
     </row>
     <row r="3" ht="13.8" customHeight="1" thickBot="1">
       <c r="A3" s="21" t="inlineStr">
@@ -2303,53 +2347,53 @@
       <c r="K3" s="22" t="n"/>
       <c r="L3" s="22" t="n"/>
       <c r="O3" s="18" t="n"/>
-      <c r="Q3" s="19" t="n"/>
       <c r="R3" s="19" t="n"/>
-      <c r="S3" s="18" t="n"/>
+      <c r="S3" s="19" t="n"/>
       <c r="T3" s="18" t="n"/>
       <c r="U3" s="18" t="n"/>
       <c r="V3" s="18" t="n"/>
       <c r="W3" s="18" t="n"/>
+      <c r="X3" s="18" t="n"/>
     </row>
     <row r="4" ht="21" customHeight="1">
-      <c r="A4" s="101" t="inlineStr">
+      <c r="A4" s="100" t="inlineStr">
         <is>
           <t xml:space="preserve">This template is for use by Product Resources to record the Process Failure Mode and Effects Analysis (DFMEA) for medical and other devices.  FMEA is also referred to as Failure Modes, Effects, and Criticality Analysis (FMECA).  </t>
         </is>
       </c>
-      <c r="B4" s="137" t="n"/>
-      <c r="C4" s="137" t="n"/>
+      <c r="B4" s="139" t="n"/>
+      <c r="C4" s="139" t="n"/>
       <c r="D4" s="18" t="n"/>
       <c r="G4" s="23" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="H4" s="95" t="inlineStr">
+      <c r="H4" s="92" t="inlineStr">
         <is>
           <t>Please see the guidance in 90-2000-7.1 regarding FMEA process before beginning an FMEA</t>
         </is>
       </c>
-      <c r="I4" s="137" t="n"/>
-      <c r="J4" s="137" t="n"/>
-      <c r="K4" s="103" t="n"/>
+      <c r="I4" s="139" t="n"/>
+      <c r="J4" s="139" t="n"/>
+      <c r="K4" s="102" t="n"/>
       <c r="L4" s="24" t="n"/>
       <c r="O4" s="18" t="n"/>
-      <c r="Q4" s="109" t="inlineStr">
+      <c r="R4" s="90" t="inlineStr">
         <is>
           <t>Parameters:</t>
         </is>
       </c>
-      <c r="R4" s="138" t="n"/>
-      <c r="S4" s="138" t="n"/>
-      <c r="T4" s="138" t="n"/>
-      <c r="U4" s="139" t="n"/>
-      <c r="V4" s="109" t="inlineStr">
+      <c r="S4" s="140" t="n"/>
+      <c r="T4" s="140" t="n"/>
+      <c r="U4" s="140" t="n"/>
+      <c r="V4" s="141" t="n"/>
+      <c r="W4" s="90" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="W4" s="139" t="n"/>
+      <c r="X4" s="141" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="19" t="n"/>
@@ -2361,27 +2405,27 @@
           <t>●</t>
         </is>
       </c>
-      <c r="H5" s="103" t="inlineStr">
+      <c r="H5" s="102" t="inlineStr">
         <is>
           <t>Initiate action to reduce the RPN</t>
         </is>
       </c>
       <c r="I5" s="19" t="n"/>
       <c r="J5" s="19" t="n"/>
-      <c r="K5" s="103" t="n"/>
+      <c r="K5" s="102" t="n"/>
       <c r="L5" s="24" t="n"/>
       <c r="O5" s="25" t="n"/>
-      <c r="Q5" s="109" t="inlineStr">
+      <c r="R5" s="90" t="inlineStr">
         <is>
           <t>RPN triggering requiring mitigation action:</t>
         </is>
       </c>
-      <c r="R5" s="138" t="n"/>
-      <c r="S5" s="138" t="n"/>
-      <c r="T5" s="138" t="n"/>
-      <c r="U5" s="138" t="n"/>
-      <c r="V5" s="139" t="n"/>
-      <c r="W5" s="26" t="n">
+      <c r="S5" s="140" t="n"/>
+      <c r="T5" s="140" t="n"/>
+      <c r="U5" s="140" t="n"/>
+      <c r="V5" s="140" t="n"/>
+      <c r="W5" s="141" t="n"/>
+      <c r="X5" s="26" t="n">
         <v>200</v>
       </c>
     </row>
@@ -2395,53 +2439,53 @@
           <t>●</t>
         </is>
       </c>
-      <c r="H6" s="103" t="inlineStr">
+      <c r="H6" s="102" t="inlineStr">
         <is>
           <t>Re-evaluate the RPN value after completion of the recommended actions</t>
         </is>
       </c>
       <c r="I6" s="19" t="n"/>
       <c r="J6" s="19" t="n"/>
-      <c r="K6" s="103" t="n"/>
+      <c r="K6" s="102" t="n"/>
       <c r="L6" s="24" t="n"/>
       <c r="O6" s="18" t="n"/>
-      <c r="Q6" s="109" t="inlineStr">
+      <c r="R6" s="90" t="inlineStr">
         <is>
           <t>Severity (Sev) requiring mitigation action regardless of RPN:</t>
         </is>
       </c>
-      <c r="R6" s="138" t="n"/>
-      <c r="S6" s="138" t="n"/>
-      <c r="T6" s="138" t="n"/>
-      <c r="U6" s="138" t="n"/>
-      <c r="V6" s="139" t="n"/>
-      <c r="W6" s="26" t="n">
+      <c r="S6" s="140" t="n"/>
+      <c r="T6" s="140" t="n"/>
+      <c r="U6" s="140" t="n"/>
+      <c r="V6" s="140" t="n"/>
+      <c r="W6" s="141" t="n"/>
+      <c r="X6" s="26" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="15.6" customHeight="1">
-      <c r="A7" s="108" t="inlineStr">
+      <c r="A7" s="89" t="inlineStr">
         <is>
           <t>PROCESS FAILURE MODE AND EFFECTS ANALYSIS (PFMEA)</t>
         </is>
       </c>
-      <c r="B7" s="138" t="n"/>
-      <c r="C7" s="138" t="n"/>
-      <c r="D7" s="138" t="n"/>
-      <c r="G7" s="138" t="n"/>
-      <c r="H7" s="138" t="n"/>
-      <c r="I7" s="138" t="n"/>
-      <c r="J7" s="138" t="n"/>
-      <c r="K7" s="138" t="n"/>
-      <c r="L7" s="138" t="n"/>
-      <c r="O7" s="138" t="n"/>
-      <c r="Q7" s="138" t="n"/>
-      <c r="R7" s="138" t="n"/>
-      <c r="S7" s="138" t="n"/>
-      <c r="T7" s="138" t="n"/>
-      <c r="U7" s="138" t="n"/>
-      <c r="V7" s="138" t="n"/>
-      <c r="W7" s="139" t="n"/>
+      <c r="B7" s="140" t="n"/>
+      <c r="C7" s="140" t="n"/>
+      <c r="D7" s="140" t="n"/>
+      <c r="G7" s="140" t="n"/>
+      <c r="H7" s="140" t="n"/>
+      <c r="I7" s="140" t="n"/>
+      <c r="J7" s="140" t="n"/>
+      <c r="K7" s="140" t="n"/>
+      <c r="L7" s="140" t="n"/>
+      <c r="O7" s="140" t="n"/>
+      <c r="R7" s="140" t="n"/>
+      <c r="S7" s="140" t="n"/>
+      <c r="T7" s="140" t="n"/>
+      <c r="U7" s="140" t="n"/>
+      <c r="V7" s="140" t="n"/>
+      <c r="W7" s="140" t="n"/>
+      <c r="X7" s="141" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
@@ -2449,43 +2493,43 @@
           <t>Item:</t>
         </is>
       </c>
-      <c r="B8" s="87" t="inlineStr">
+      <c r="B8" s="98" t="inlineStr">
         <is>
           <t>Wheel damper</t>
         </is>
       </c>
-      <c r="C8" s="138" t="n"/>
-      <c r="D8" s="139" t="n"/>
+      <c r="C8" s="140" t="n"/>
+      <c r="D8" s="141" t="n"/>
       <c r="G8" s="28" t="n"/>
-      <c r="H8" s="88" t="inlineStr">
+      <c r="H8" s="108" t="inlineStr">
         <is>
           <t>Responsibility:</t>
         </is>
       </c>
-      <c r="I8" s="138" t="n"/>
-      <c r="J8" s="139" t="n"/>
-      <c r="K8" s="87" t="inlineStr">
+      <c r="I8" s="140" t="n"/>
+      <c r="J8" s="141" t="n"/>
+      <c r="K8" s="98" t="inlineStr">
         <is>
           <t>Donald Trump</t>
         </is>
       </c>
-      <c r="L8" s="138" t="n"/>
-      <c r="O8" s="139" t="n"/>
-      <c r="Q8" s="28" t="n"/>
-      <c r="R8" s="27" t="inlineStr">
+      <c r="L8" s="140" t="n"/>
+      <c r="O8" s="141" t="n"/>
+      <c r="R8" s="28" t="n"/>
+      <c r="S8" s="27" t="inlineStr">
         <is>
           <t>FMEA number:</t>
         </is>
       </c>
-      <c r="S8" s="87" t="inlineStr">
+      <c r="T8" s="98" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
       </c>
-      <c r="T8" s="138" t="n"/>
-      <c r="U8" s="138" t="n"/>
-      <c r="V8" s="138" t="n"/>
-      <c r="W8" s="139" t="n"/>
+      <c r="U8" s="140" t="n"/>
+      <c r="V8" s="140" t="n"/>
+      <c r="W8" s="140" t="n"/>
+      <c r="X8" s="141" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
@@ -2493,39 +2537,39 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="B9" s="87" t="inlineStr">
+      <c r="B9" s="98" t="inlineStr">
         <is>
           <t>Drive shaft</t>
         </is>
       </c>
-      <c r="C9" s="138" t="n"/>
-      <c r="D9" s="139" t="n"/>
-      <c r="G9" s="86" t="n"/>
-      <c r="H9" s="100" t="inlineStr">
+      <c r="C9" s="140" t="n"/>
+      <c r="D9" s="141" t="n"/>
+      <c r="G9" s="107" t="n"/>
+      <c r="H9" s="99" t="inlineStr">
         <is>
           <t>Prepared by:</t>
         </is>
       </c>
-      <c r="I9" s="138" t="n"/>
-      <c r="J9" s="139" t="n"/>
-      <c r="K9" s="87" t="inlineStr">
+      <c r="I9" s="140" t="n"/>
+      <c r="J9" s="141" t="n"/>
+      <c r="K9" s="98" t="inlineStr">
         <is>
           <t>Selva Jeyaseelan</t>
         </is>
       </c>
-      <c r="L9" s="138" t="n"/>
-      <c r="O9" s="139" t="n"/>
-      <c r="Q9" s="28" t="n"/>
-      <c r="R9" s="27" t="inlineStr">
+      <c r="L9" s="140" t="n"/>
+      <c r="O9" s="141" t="n"/>
+      <c r="R9" s="28" t="n"/>
+      <c r="S9" s="27" t="inlineStr">
         <is>
           <t>Page :</t>
         </is>
       </c>
-      <c r="S9" s="86" t="n"/>
-      <c r="T9" s="138" t="n"/>
-      <c r="U9" s="138" t="n"/>
-      <c r="V9" s="138" t="n"/>
-      <c r="W9" s="139" t="n"/>
+      <c r="T9" s="107" t="n"/>
+      <c r="U9" s="140" t="n"/>
+      <c r="V9" s="140" t="n"/>
+      <c r="W9" s="140" t="n"/>
+      <c r="X9" s="141" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
@@ -2533,37 +2577,37 @@
           <t>Core Team:</t>
         </is>
       </c>
-      <c r="B10" s="104" t="inlineStr">
+      <c r="B10" s="103" t="inlineStr">
         <is>
           <t>Sunder Pichai, Sam Altman, Selva Jeyaseelan</t>
         </is>
       </c>
-      <c r="C10" s="138" t="n"/>
-      <c r="D10" s="138" t="n"/>
-      <c r="G10" s="138" t="n"/>
-      <c r="H10" s="138" t="n"/>
-      <c r="I10" s="138" t="n"/>
-      <c r="J10" s="138" t="n"/>
-      <c r="K10" s="138" t="n"/>
-      <c r="L10" s="138" t="n"/>
-      <c r="O10" s="139" t="n"/>
-      <c r="Q10" s="28" t="n"/>
-      <c r="R10" s="27" t="inlineStr">
+      <c r="C10" s="140" t="n"/>
+      <c r="D10" s="140" t="n"/>
+      <c r="G10" s="140" t="n"/>
+      <c r="H10" s="140" t="n"/>
+      <c r="I10" s="140" t="n"/>
+      <c r="J10" s="140" t="n"/>
+      <c r="K10" s="140" t="n"/>
+      <c r="L10" s="140" t="n"/>
+      <c r="O10" s="141" t="n"/>
+      <c r="R10" s="28" t="n"/>
+      <c r="S10" s="27" t="inlineStr">
         <is>
           <t>FMEA Date (Orig):</t>
         </is>
       </c>
-      <c r="S10" s="30" t="n">
+      <c r="T10" s="30" t="n">
         <v>46270</v>
       </c>
-      <c r="T10" s="91" t="inlineStr">
+      <c r="U10" s="109" t="inlineStr">
         <is>
           <t>Rev:</t>
         </is>
       </c>
-      <c r="U10" s="139" t="n"/>
-      <c r="V10" s="92" t="n"/>
-      <c r="W10" s="139" t="n"/>
+      <c r="V10" s="141" t="n"/>
+      <c r="W10" s="110" t="n"/>
+      <c r="X10" s="141" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="28" t="n"/>
@@ -2577,196 +2621,201 @@
       <c r="K11" s="28" t="n"/>
       <c r="L11" s="28" t="n"/>
       <c r="O11" s="31" t="n"/>
-      <c r="Q11" s="28" t="n"/>
-      <c r="R11" s="27" t="inlineStr">
+      <c r="R11" s="28" t="n"/>
+      <c r="S11" s="27" t="inlineStr">
         <is>
           <t>FMEA Date (Cur):</t>
         </is>
       </c>
-      <c r="S11" s="30" t="n">
+      <c r="T11" s="30" t="n">
         <v>46270</v>
       </c>
-      <c r="T11" s="91" t="inlineStr">
+      <c r="U11" s="109" t="inlineStr">
         <is>
           <t>Rev:</t>
         </is>
       </c>
-      <c r="U11" s="139" t="n"/>
-      <c r="V11" s="92" t="n"/>
-      <c r="W11" s="139" t="n"/>
+      <c r="V11" s="141" t="n"/>
+      <c r="W11" s="110" t="n"/>
+      <c r="X11" s="141" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="140" t="inlineStr">
+      <c r="A12" s="142" t="inlineStr">
         <is>
           <t xml:space="preserve"> Process</t>
         </is>
       </c>
-      <c r="B12" s="90" t="inlineStr">
+      <c r="B12" s="85" t="inlineStr">
         <is>
           <t>Potential Failure Mode</t>
         </is>
       </c>
-      <c r="C12" s="90" t="inlineStr">
+      <c r="C12" s="85" t="inlineStr">
         <is>
           <t>Potential Effect(s) of Failure</t>
         </is>
       </c>
-      <c r="D12" s="89" t="inlineStr">
+      <c r="D12" s="95" t="inlineStr">
         <is>
           <t>Sev</t>
         </is>
       </c>
-      <c r="E12" s="141" t="inlineStr">
+      <c r="E12" s="143" t="inlineStr">
         <is>
           <t>pred sev</t>
         </is>
       </c>
-      <c r="F12" s="141" t="inlineStr">
+      <c r="F12" s="143" t="inlineStr">
         <is>
           <t>sev reasoning</t>
         </is>
       </c>
-      <c r="G12" s="89" t="inlineStr">
+      <c r="G12" s="95" t="inlineStr">
         <is>
           <t>Cls</t>
         </is>
       </c>
-      <c r="H12" s="90" t="inlineStr">
+      <c r="H12" s="85" t="inlineStr">
         <is>
           <t>Potential Cause(s)/ Mechanism(s) of Failure</t>
         </is>
       </c>
-      <c r="I12" s="90" t="inlineStr">
+      <c r="I12" s="85" t="inlineStr">
         <is>
           <t>Current 
 Process Prevention
 Controls</t>
         </is>
       </c>
-      <c r="J12" s="89" t="inlineStr">
+      <c r="J12" s="95" t="inlineStr">
         <is>
           <t>Occ</t>
         </is>
       </c>
-      <c r="K12" s="90" t="inlineStr">
+      <c r="K12" s="85" t="inlineStr">
         <is>
           <t>Current 
 Process Detection Controls
 Controls</t>
         </is>
       </c>
-      <c r="L12" s="89" t="inlineStr">
+      <c r="L12" s="95" t="inlineStr">
         <is>
           <t>Det</t>
         </is>
       </c>
-      <c r="M12" s="141" t="inlineStr">
+      <c r="M12" s="143" t="inlineStr">
         <is>
           <t>pred det</t>
         </is>
       </c>
-      <c r="N12" s="141" t="inlineStr">
+      <c r="N12" s="143" t="inlineStr">
         <is>
           <t>det reasoning</t>
         </is>
       </c>
-      <c r="O12" s="89" t="inlineStr">
+      <c r="O12" s="95" t="inlineStr">
         <is>
           <t>RPN</t>
         </is>
       </c>
-      <c r="P12" s="141" t="inlineStr">
+      <c r="P12" s="143" t="inlineStr">
         <is>
           <t>D-P gap</t>
         </is>
       </c>
-      <c r="Q12" s="90" t="inlineStr">
+      <c r="R12" s="85" t="inlineStr">
         <is>
           <t>Recommended Action(s)</t>
         </is>
       </c>
-      <c r="R12" s="90" t="inlineStr">
+      <c r="S12" s="85" t="inlineStr">
         <is>
           <t>Responsibility and Target Completion Date</t>
         </is>
       </c>
-      <c r="S12" s="93" t="inlineStr">
+      <c r="T12" s="111" t="inlineStr">
         <is>
           <t>Action Results</t>
         </is>
       </c>
-      <c r="T12" s="138" t="n"/>
-      <c r="U12" s="138" t="n"/>
-      <c r="V12" s="138" t="n"/>
-      <c r="W12" s="139" t="n"/>
+      <c r="U12" s="140" t="n"/>
+      <c r="V12" s="140" t="n"/>
+      <c r="W12" s="140" t="n"/>
+      <c r="X12" s="141" t="n"/>
     </row>
     <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="142" t="n"/>
-      <c r="B13" s="142" t="n"/>
-      <c r="C13" s="142" t="n"/>
-      <c r="D13" s="142" t="n"/>
-      <c r="E13" s="143" t="n"/>
-      <c r="F13" s="143" t="n"/>
-      <c r="G13" s="142" t="n"/>
-      <c r="H13" s="142" t="n"/>
-      <c r="I13" s="142" t="n"/>
-      <c r="J13" s="142" t="n"/>
-      <c r="K13" s="142" t="n"/>
-      <c r="L13" s="142" t="n"/>
-      <c r="M13" s="143" t="n"/>
-      <c r="N13" s="143" t="n"/>
-      <c r="O13" s="142" t="n"/>
-      <c r="P13" s="143" t="n"/>
-      <c r="Q13" s="142" t="n"/>
-      <c r="R13" s="142" t="n"/>
-      <c r="S13" s="90" t="inlineStr">
+      <c r="A13" s="144" t="n"/>
+      <c r="B13" s="144" t="n"/>
+      <c r="C13" s="144" t="n"/>
+      <c r="D13" s="144" t="n"/>
+      <c r="E13" s="145" t="n"/>
+      <c r="F13" s="145" t="n"/>
+      <c r="G13" s="144" t="n"/>
+      <c r="H13" s="144" t="n"/>
+      <c r="I13" s="144" t="n"/>
+      <c r="J13" s="144" t="n"/>
+      <c r="K13" s="144" t="n"/>
+      <c r="L13" s="144" t="n"/>
+      <c r="M13" s="145" t="n"/>
+      <c r="N13" s="145" t="n"/>
+      <c r="O13" s="144" t="n"/>
+      <c r="P13" s="145" t="n"/>
+      <c r="R13" s="144" t="n"/>
+      <c r="S13" s="144" t="n"/>
+      <c r="T13" s="85" t="inlineStr">
         <is>
           <t>Actions Taken</t>
         </is>
       </c>
-      <c r="T13" s="89" t="inlineStr">
+      <c r="U13" s="95" t="inlineStr">
         <is>
           <t>Sev</t>
         </is>
       </c>
-      <c r="U13" s="89" t="inlineStr">
+      <c r="V13" s="95" t="inlineStr">
         <is>
           <t>Occ</t>
         </is>
       </c>
-      <c r="V13" s="89" t="inlineStr">
+      <c r="W13" s="95" t="inlineStr">
         <is>
           <t>Det</t>
         </is>
       </c>
-      <c r="W13" s="89" t="inlineStr">
+      <c r="X13" s="95" t="inlineStr">
         <is>
           <t>RPN</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="118.8" customHeight="1">
-      <c r="A14" s="85" t="n"/>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>More grease in the bearning</t>
+    <row r="14" ht="92.40000000000001" customHeight="1">
+      <c r="A14" s="146" t="inlineStr">
+        <is>
+          <t>10. Grease plastic bearning</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>No grease filled in the bearing</t>
         </is>
       </c>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
-OEM: Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning(9)</t>
+          <t>S: Portion of production run may have to be scrapped (7)
+OEM: Portion of production run may have to be scrapped (7)
+EU: Degradtion of primary function (7)</t>
         </is>
       </c>
       <c r="D14" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E14" s="144" t="n">
-        <v>9</v>
-      </c>
-      <c r="F14" s="145" t="inlineStr">
-        <is>
-          <t>failure effect text keywords do not match AIAG severity definition. OEM effect does not semantically match severity 9 because it states safe operation/regulatory noncompliance with warning, which is consistent with 9; however the S effect states reworked off line and accepted, which is consistent with 6, not 5. Recommended Severity: 9</t>
+        <v>7</v>
+      </c>
+      <c r="E14" s="147" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="148" t="inlineStr">
+        <is>
+          <t>severity is correct</t>
         </is>
       </c>
       <c r="G14" s="13" t="n"/>
@@ -2787,129 +2836,697 @@
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
+          <t>Read switch to find the level of grease in the tank (2)
+Layer Process Audit (6)</t>
+        </is>
+      </c>
+      <c r="L14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="147" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="148" t="inlineStr">
+        <is>
+          <t>detection controls text matches AIAG detection criteria</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="P14" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R14" s="13" t="n"/>
+      <c r="S14" s="13" t="n"/>
+      <c r="T14" s="14" t="n"/>
+      <c r="U14" s="14" t="n"/>
+      <c r="V14" s="14" t="n"/>
+      <c r="W14" s="14" t="n"/>
+      <c r="X14" s="2">
+        <f>IF(O14*P14*Q14&gt;0,O14*P14*Q14,K14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="79.2" customHeight="1">
+      <c r="A15" s="150" t="n"/>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Less grease in the bearing</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S: Portion of production run may have to be scrapped (5)
+OEM: Portion of production run may have to be scrapped (7)
+</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="151" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="152" t="inlineStr">
+        <is>
+          <t>'Portion of production run may have to be scrapped' maps to AIAG 7. The stated severity 5 is an under-rating.</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Severity test: Lower severity choosen</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Preventive maintenance
+Calibration of gage</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
           <t>First Off Approval (2)
 Layered Process Audit (6)
 Calibration report (6)</t>
         </is>
       </c>
-      <c r="L14" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="M14" s="144" t="n">
+      <c r="M15" s="151" t="n">
         <v>2</v>
       </c>
-      <c r="N14" s="145" t="inlineStr">
-        <is>
-          <t>detection controls text keywords do not match AIAG detection criteria. Check 1 failed: Original Stated Detection does not exactly match Strongest Detection Extracted. Recommended Detection: 2</t>
-        </is>
-      </c>
-      <c r="O14" s="2">
-        <f>D14*H14*J14</f>
-        <v/>
-      </c>
-      <c r="P14" s="146" t="inlineStr">
+      <c r="N15" s="152" t="inlineStr">
+        <is>
+          <t>detection controls text keywords do not match AIAG detection criteria. Check 1 failed: Original Stated Detection (5) does not exactly match Strongest Detection Extracted (2). Recommended Detection: 2</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="P15" s="149" t="inlineStr">
         <is>
           <t>no gap</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="n"/>
-      <c r="R14" s="13" t="n"/>
-      <c r="S14" s="14" t="n"/>
-      <c r="T14" s="14" t="n"/>
-      <c r="U14" s="14" t="n"/>
-      <c r="V14" s="14" t="n"/>
-      <c r="W14" s="2">
-        <f>IF(O14*P14*Q14&gt;0,O14*P14*Q14,K14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="118.8" customHeight="1">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="13" t="n"/>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
-OEM: Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning(9)</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E15" s="144" t="n">
-        <v>9</v>
-      </c>
-      <c r="F15" s="145" t="inlineStr">
-        <is>
-          <t>failure effect text keywords do not match AIAG severity definition. Check 2 failed: the (5) effect describes rework off line and accepted, which matches Severity 6, not 5. Recommended Severity: 9</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="16" t="inlineStr">
-        <is>
-          <t>DFMEA PFMEA Gap analysis check</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>Detection test scenario: Multiple Controls (Stated matches Weakest)</t>
-        </is>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="13" t="inlineStr">
-        <is>
-          <t>"Visual check by operator (8) \n Automated laser interlock in-station (3)"</t>
-        </is>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="M15" s="144" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" s="145" t="inlineStr">
-        <is>
-          <t>detection controls text keywords do not match AIAG detection criteria. Check 1 failed: Original Stated Detection (8) does not exactly match Strongest Detection Extracted (3). Recommended Detection: 3</t>
-        </is>
-      </c>
-      <c r="O15" s="2">
-        <f>D15*H15*J15</f>
-        <v/>
-      </c>
-      <c r="P15" s="146" t="inlineStr">
-        <is>
-          <t>no gap</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="n"/>
       <c r="R15" s="13" t="n"/>
-      <c r="S15" s="14" t="n"/>
+      <c r="S15" s="13" t="n"/>
       <c r="T15" s="14" t="n"/>
       <c r="U15" s="14" t="n"/>
       <c r="V15" s="14" t="n"/>
-      <c r="W15" s="2">
+      <c r="W15" s="14" t="n"/>
+      <c r="X15" s="2">
         <f>IF(O15*P15*Q15&gt;0,O15*P15*Q15,K15)</f>
         <v/>
       </c>
     </row>
+    <row r="16" ht="118.8" customHeight="1">
+      <c r="A16" s="144" t="n"/>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>More grease in the bearning</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
+OEM: Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning(9)</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="147" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="148" t="inlineStr">
+        <is>
+          <t>severity is correct</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n"/>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Severity Test:Defect text matches AIAG standard</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Daily maintenace check sheet
+Preventive Maintenance
+Work instruction for grease refill</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>First Off Approval (2)
+Layered Process Audit (6)
+Calibration report (6)</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="M16" s="151" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" s="152" t="inlineStr">
+        <is>
+          <t>detection controls text keywords do not match AIAG detection criteria. Check 1 failed: Original Stated Detection (5) does not exactly match Strongest Detection Extracted (2). Recommended Detection: 2</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="P16" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R16" s="13" t="n"/>
+      <c r="S16" s="13" t="n"/>
+      <c r="T16" s="14" t="n"/>
+      <c r="U16" s="14" t="n"/>
+      <c r="V16" s="14" t="n"/>
+      <c r="W16" s="14" t="n"/>
+      <c r="X16" s="2">
+        <f>IF(O16*P16*Q16&gt;0,O16*P16*Q16,K16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="105.6" customHeight="1">
+      <c r="A17" s="13" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
+OEM: No discernible effect (1)</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="151" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="152" t="inlineStr">
+        <is>
+          <t>"A proportion of the production run may have to be reworked off line and accepted" maps to AIAG severity 6. The stated severity 5 is an under-rating.</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n"/>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Severity test scenario: perfect match</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Severe Semantic Mismatch (Over-rating)</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>"Random visual inspection by supervisor once a shift (3)"</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" s="151" t="n">
+        <v>9</v>
+      </c>
+      <c r="N17" s="152" t="inlineStr">
+        <is>
+          <t>detection controls text keywords do not match AIAG detection criteria. Check 2 failed: "Random visual inspection by supervisor once a shift (3)" describes a weak random audit/visual inspection, not AIAG detection level 3. Recommended Detection: 9</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="P17" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="n"/>
+      <c r="S17" s="13" t="n"/>
+      <c r="T17" s="14" t="n"/>
+      <c r="U17" s="14" t="n"/>
+      <c r="V17" s="14" t="n"/>
+      <c r="W17" s="14" t="n"/>
+      <c r="X17" s="2">
+        <f>IF(O17*P17*Q17&gt;0,O17*P17*Q17,K17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="79.2" customHeight="1">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>EU: Apperance, fit and finish type itms do not confrm, defect noticed by most of the customrs (&gt;75%) (4)</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="147" t="n">
+        <v>4</v>
+      </c>
+      <c r="F18" s="148" t="inlineStr">
+        <is>
+          <t>severity is correct</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n"/>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Severity test scenario: Spelling and typo</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Severe Semantic Mismatch (Under-rating)</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>"In-station automated vision system that locks the machine if a defect is found (8)"</t>
+        </is>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="M18" s="151" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="152" t="inlineStr">
+        <is>
+          <t>detection controls text keywords do not match AIAG detection criteria. The text describes in-station automated lock/stop control, which aligns to AIAG 3, not 8. Recommended Detection: 3</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="P18" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R18" s="13" t="n"/>
+      <c r="S18" s="13" t="n"/>
+      <c r="T18" s="14" t="n"/>
+      <c r="U18" s="14" t="n"/>
+      <c r="V18" s="14" t="n"/>
+      <c r="W18" s="14" t="n"/>
+      <c r="X18" s="2">
+        <f>IF(O18*P18*Q18&gt;0,O18*P18*Q18,K18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="105.6" customHeight="1">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="n"/>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>S: 100% of product may have to be scrapped. Line shutdown or stop ship. (8)
+OEM: A portion of the production run may have to be scrapped. (7)</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" s="151" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" s="152" t="inlineStr">
+        <is>
+          <t>'100% of product may have to be scrapped. Line shutdown or stop ship.' maps to AIAG 8, which is higher than the stated severity 7.</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="n"/>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Severity test scenario: Column Mismatch (Under-reporting)</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Heavy Typographical Errors</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>"Aoutmated varible gaging with red light buzer to notfy opreator (5)"</t>
+        </is>
+      </c>
+      <c r="L19" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="147" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="148" t="inlineStr">
+        <is>
+          <t>detection controls text matches AIAG detection criteria</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="P19" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="n"/>
+      <c r="S19" s="13" t="n"/>
+      <c r="T19" s="14" t="n"/>
+      <c r="U19" s="14" t="n"/>
+      <c r="V19" s="14" t="n"/>
+      <c r="W19" s="14" t="n"/>
+      <c r="X19" s="2">
+        <f>IF(O19*P19*Q19&gt;0,O19*P19*Q19,K19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="66" customHeight="1">
+      <c r="A20" s="13" t="n"/>
+      <c r="B20" s="13" t="n"/>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Mismatch	EU: Loss of primary function (product inoperable, does not affect safe operation) (4)</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" s="151" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="152" t="inlineStr">
+        <is>
+          <t>'Loss of primary function' maps to AIAG 8. The stated 4 is an under-rating.</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="n"/>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Severity test scenario: EU: Loss of primary function (product inoperable, does not affect safe operation) (4)</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Detection test scenario: . Multiple Controls (Stated matches Strongest)</t>
+        </is>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>"Visual check by operator (8)  Automated laser interlock in-station (3)"</t>
+        </is>
+      </c>
+      <c r="L20" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" s="147" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="148" t="inlineStr">
+        <is>
+          <t>detection controls text matches AIAG detection criteria</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="P20" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="n"/>
+      <c r="S20" s="13" t="n"/>
+      <c r="T20" s="14" t="n"/>
+      <c r="U20" s="14" t="n"/>
+      <c r="V20" s="14" t="n"/>
+      <c r="W20" s="14" t="n"/>
+      <c r="X20" s="2">
+        <f>IF(O20*P20*Q20&gt;0,O20*P20*Q20,K20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="118.8" customHeight="1">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
+OEM: Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning(9)</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" s="147" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="148" t="inlineStr">
+        <is>
+          <t>severity is correct</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="n"/>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>DFMEA PFMEA Gap analysis check</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Multiple Controls (Stated matches Weakest)</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>"Visual check by operator (8) \n Automated laser interlock in-station (3)"</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="M21" s="151" t="n">
+        <v>3</v>
+      </c>
+      <c r="N21" s="152" t="inlineStr">
+        <is>
+          <t>detection controls text keywords do not match AIAG detection criteria. Check 1 failed: Original Stated Detection (8) does not exactly match Strongest Detection Extracted (3). Recommended Detection: 3</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>216</v>
+      </c>
+      <c r="P21" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R21" s="13" t="n"/>
+      <c r="S21" s="13" t="n"/>
+      <c r="T21" s="14" t="n"/>
+      <c r="U21" s="14" t="n"/>
+      <c r="V21" s="14" t="n"/>
+      <c r="W21" s="14" t="n"/>
+      <c r="X21" s="2">
+        <f>IF(O21*P21*Q21&gt;0,O21*P21*Q21,K21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="118.8" customHeight="1">
+      <c r="A22" s="13" t="n"/>
+      <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>S: A proportion of the production run may have to be reworked off line and accepted (5)
+OEM: Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning(9)</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E22" s="151" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="152" t="inlineStr">
+        <is>
+          <t>'Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning' maps to AIAG 9, which is the highest effect described.</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n"/>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>DFMEA PFMEA Gap analysis check</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Missing Brackets / Parentheses</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>"Manual attribute go/no-go gauging in station 7"</t>
+        </is>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="M22" s="147" t="n">
+        <v>7</v>
+      </c>
+      <c r="N22" s="148" t="inlineStr">
+        <is>
+          <t>detection controls text matches AIAG detection criteria</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="P22" s="153" t="inlineStr">
+        <is>
+          <t>Gap identified. Det must be &lt;3</t>
+        </is>
+      </c>
+      <c r="R22" s="13" t="n"/>
+      <c r="S22" s="13" t="n"/>
+      <c r="T22" s="14" t="n"/>
+      <c r="U22" s="14" t="n"/>
+      <c r="V22" s="14" t="n"/>
+      <c r="W22" s="14" t="n"/>
+      <c r="X22" s="2">
+        <f>IF(O22*P22*Q22&gt;0,O22*P22*Q22,K22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="92.40000000000001" customHeight="1">
+      <c r="A23" s="13" t="n"/>
+      <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>S: Portion of production run may have to be scrapped (7)
+OEM: Portion of production run may have to be scrapped (7)
+EU: Degradtion of primary function (7)</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" s="147" t="n">
+        <v>7</v>
+      </c>
+      <c r="F23" s="148" t="inlineStr">
+        <is>
+          <t>severity is correct</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="n"/>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Severity Test:Defect text matches AIAG standard</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>Detection test scenario: Number Confusions (Scores mixed with specs)</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>"Check 5 times a day using a 2 mm variable gauge (6)"`</t>
+        </is>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" s="147" t="n">
+        <v>6</v>
+      </c>
+      <c r="N23" s="148" t="inlineStr">
+        <is>
+          <t>detection controls text matches AIAG detection criteria</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="P23" s="149" t="inlineStr">
+        <is>
+          <t>no gap</t>
+        </is>
+      </c>
+      <c r="R23" s="13" t="n"/>
+      <c r="S23" s="13" t="n"/>
+      <c r="T23" s="14" t="n"/>
+      <c r="U23" s="14" t="n"/>
+      <c r="V23" s="14" t="n"/>
+      <c r="W23" s="14" t="n"/>
+      <c r="X23" s="2">
+        <f>IF(O23*P23*Q23&gt;0,O23*P23*Q23,K23)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
+    <mergeCell ref="W4:X4"/>
+    <mergeCell ref="R6:W6"/>
+    <mergeCell ref="A7:X7"/>
     <mergeCell ref="B12:B13"/>
-    <mergeCell ref="S12:W12"/>
-    <mergeCell ref="Q5:V5"/>
+    <mergeCell ref="W10:X10"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="F12:F13"/>
     <mergeCell ref="L12:L13"/>
     <mergeCell ref="N12:N13"/>
     <mergeCell ref="K9:O9"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Q6:V6"/>
-    <mergeCell ref="S8:W8"/>
-    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="R4:V4"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="R12:R13"/>
-    <mergeCell ref="V10:W10"/>
+    <mergeCell ref="U11:V11"/>
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="I12:I13"/>
     <mergeCell ref="K12:K13"/>
@@ -2917,40 +3534,51 @@
     <mergeCell ref="M12:M13"/>
     <mergeCell ref="O12:O13"/>
     <mergeCell ref="D12:D13"/>
-    <mergeCell ref="A7:W7"/>
-    <mergeCell ref="Q4:U4"/>
-    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="T9:X9"/>
+    <mergeCell ref="T12:X12"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="K8:O8"/>
-    <mergeCell ref="V11:W11"/>
     <mergeCell ref="H12:H13"/>
+    <mergeCell ref="R5:W5"/>
     <mergeCell ref="B10:O10"/>
     <mergeCell ref="H8:J8"/>
     <mergeCell ref="J12:J13"/>
     <mergeCell ref="A4:C6"/>
     <mergeCell ref="P12:P13"/>
-    <mergeCell ref="S9:W9"/>
+    <mergeCell ref="T8:X8"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="W11:X11"/>
     <mergeCell ref="E12:E13"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="H4:J4"/>
-    <mergeCell ref="Q12:Q13"/>
+    <mergeCell ref="U10:V10"/>
     <mergeCell ref="H9:J9"/>
+    <mergeCell ref="S12:S13"/>
     <mergeCell ref="H6:J6"/>
   </mergeCells>
-  <conditionalFormatting sqref="D14:D15 K14:K15 O14:O15 R14:R15">
+  <conditionalFormatting sqref="D14:D23 R14:R23">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K14:K23">
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O14:O23">
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="0" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="D14:D15 O14:O15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="D14:D23 O14:O23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Sev</formula1>
     </dataValidation>
-    <dataValidation sqref="H14:H15 P14:P15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="H14:H23 P14:P23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Occur</formula1>
     </dataValidation>
-    <dataValidation sqref="J14:J15 Q14:Q15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J14:J23 Q14:Q23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Det</formula1>
     </dataValidation>
   </dataValidations>
@@ -2990,48 +3618,48 @@
       </c>
     </row>
     <row r="2" ht="39" customHeight="1" thickBot="1">
-      <c r="B2" s="147" t="inlineStr">
+      <c r="B2" s="154" t="inlineStr">
         <is>
           <t>PFMEA - Detection
 The team should agree on the criteria and ranking values. Select one way and consistently apply that scale.</t>
         </is>
       </c>
-      <c r="C2" s="148" t="n"/>
-      <c r="D2" s="148" t="n"/>
-      <c r="E2" s="148" t="n"/>
-      <c r="F2" s="148" t="n"/>
-      <c r="G2" s="148" t="n"/>
-      <c r="H2" s="149" t="n"/>
+      <c r="C2" s="155" t="n"/>
+      <c r="D2" s="155" t="n"/>
+      <c r="E2" s="155" t="n"/>
+      <c r="F2" s="155" t="n"/>
+      <c r="G2" s="155" t="n"/>
+      <c r="H2" s="156" t="n"/>
       <c r="I2" s="74" t="n"/>
     </row>
     <row r="3" ht="18.6" customHeight="1" thickBot="1">
-      <c r="B3" s="132" t="inlineStr">
+      <c r="B3" s="134" t="inlineStr">
         <is>
           <t>References</t>
         </is>
       </c>
-      <c r="C3" s="132" t="inlineStr">
+      <c r="C3" s="134" t="inlineStr">
         <is>
           <t>Modified from J1739 / AS13004</t>
         </is>
       </c>
-      <c r="D3" s="149" t="n"/>
-      <c r="E3" s="122" t="inlineStr">
+      <c r="D3" s="156" t="n"/>
+      <c r="E3" s="124" t="inlineStr">
         <is>
           <t xml:space="preserve"> Mistake-proofed</t>
         </is>
       </c>
-      <c r="F3" s="122" t="inlineStr">
+      <c r="F3" s="124" t="inlineStr">
         <is>
           <t xml:space="preserve"> Gauged</t>
         </is>
       </c>
-      <c r="G3" s="122" t="inlineStr">
+      <c r="G3" s="124" t="inlineStr">
         <is>
           <t xml:space="preserve"> Manual Inspection  </t>
         </is>
       </c>
-      <c r="H3" s="122" t="inlineStr">
+      <c r="H3" s="124" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -3039,25 +3667,25 @@
       <c r="I3" s="74" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1" thickBot="1">
-      <c r="B4" s="122" t="inlineStr">
+      <c r="B4" s="124" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="C4" s="122" t="inlineStr">
+      <c r="C4" s="124" t="inlineStr">
         <is>
           <t>Likelihood of Detection by Process Control - Category</t>
         </is>
       </c>
-      <c r="D4" s="122" t="inlineStr">
+      <c r="D4" s="124" t="inlineStr">
         <is>
           <t>Likelihood of Detection by Process Control - Criteria</t>
         </is>
       </c>
-      <c r="E4" s="150" t="n"/>
-      <c r="F4" s="150" t="n"/>
-      <c r="G4" s="150" t="n"/>
-      <c r="H4" s="150" t="n"/>
+      <c r="E4" s="157" t="n"/>
+      <c r="F4" s="157" t="n"/>
+      <c r="G4" s="157" t="n"/>
+      <c r="H4" s="157" t="n"/>
       <c r="K4" s="75" t="n"/>
     </row>
     <row r="5" ht="42" customHeight="1" thickBot="1">
@@ -3076,7 +3704,7 @@
       </c>
       <c r="E5" s="77" t="n"/>
       <c r="F5" s="78" t="n"/>
-      <c r="G5" s="151" t="inlineStr">
+      <c r="G5" s="158" t="inlineStr">
         <is>
           <t xml:space="preserve">100% Human Inspection </t>
         </is>
@@ -3099,7 +3727,7 @@
       </c>
       <c r="E6" s="80" t="n"/>
       <c r="F6" s="78" t="n"/>
-      <c r="G6" s="152" t="n"/>
+      <c r="G6" s="159" t="n"/>
       <c r="H6" s="79" t="n"/>
     </row>
     <row r="7" ht="42" customHeight="1" thickBot="1">
@@ -3118,7 +3746,7 @@
       </c>
       <c r="E7" s="80" t="n"/>
       <c r="F7" s="78" t="n"/>
-      <c r="G7" s="152" t="n"/>
+      <c r="G7" s="159" t="n"/>
       <c r="H7" s="79" t="n"/>
     </row>
     <row r="8" ht="42" customHeight="1" thickBot="1">
@@ -3136,12 +3764,12 @@
         </is>
       </c>
       <c r="E8" s="80" t="n"/>
-      <c r="F8" s="151" t="inlineStr">
+      <c r="F8" s="158" t="inlineStr">
         <is>
           <t>Manual gauging is used on every part</t>
         </is>
       </c>
-      <c r="G8" s="152" t="n"/>
+      <c r="G8" s="159" t="n"/>
       <c r="H8" s="79" t="n"/>
     </row>
     <row r="9" ht="42" customHeight="1" thickBot="1">
@@ -3159,8 +3787,8 @@
         </is>
       </c>
       <c r="E9" s="80" t="n"/>
-      <c r="F9" s="150" t="n"/>
-      <c r="G9" s="152" t="n"/>
+      <c r="F9" s="157" t="n"/>
+      <c r="G9" s="159" t="n"/>
       <c r="H9" s="79" t="n"/>
     </row>
     <row r="10" ht="58.5" customHeight="1" thickBot="1">
@@ -3178,12 +3806,12 @@
         </is>
       </c>
       <c r="E10" s="80" t="n"/>
-      <c r="F10" s="151" t="inlineStr">
+      <c r="F10" s="158" t="inlineStr">
         <is>
           <t>Automatic gauging or controls to detect discrepant part</t>
         </is>
       </c>
-      <c r="G10" s="150" t="n"/>
+      <c r="G10" s="157" t="n"/>
       <c r="H10" s="79" t="n"/>
     </row>
     <row r="11" ht="42" customHeight="1" thickBot="1">
@@ -3200,12 +3828,12 @@
           <t>Defect (Failure Mode) detection post-processing by automated controls that will detect discrepant part and lock part to prevent further processing.</t>
         </is>
       </c>
-      <c r="E11" s="151" t="inlineStr">
+      <c r="E11" s="158" t="inlineStr">
         <is>
           <t>Controls in place for mistake proofing the assembly</t>
         </is>
       </c>
-      <c r="F11" s="152" t="n"/>
+      <c r="F11" s="159" t="n"/>
       <c r="G11" s="81" t="n"/>
       <c r="H11" s="79" t="n"/>
     </row>
@@ -3223,8 +3851,8 @@
           <t>Defect (Failure Mode) detection in-station by automated controls that will detect discrepant part and automatically lock part in station to prevent further processing.</t>
         </is>
       </c>
-      <c r="E12" s="152" t="n"/>
-      <c r="F12" s="150" t="n"/>
+      <c r="E12" s="159" t="n"/>
+      <c r="F12" s="157" t="n"/>
       <c r="G12" s="81" t="n"/>
       <c r="H12" s="79" t="n"/>
     </row>
@@ -3242,7 +3870,7 @@
           <t>Error (Cause) detection in-station by automated controls that will detect error and prevent discrepant part from being made.</t>
         </is>
       </c>
-      <c r="E13" s="152" t="n"/>
+      <c r="E13" s="159" t="n"/>
       <c r="F13" s="78" t="n"/>
       <c r="G13" s="81" t="n"/>
       <c r="H13" s="79" t="n"/>
@@ -3261,7 +3889,7 @@
           <t>Error (Cause) prevention as a result of fixture design, machine design or part design.</t>
         </is>
       </c>
-      <c r="E14" s="150" t="n"/>
+      <c r="E14" s="157" t="n"/>
       <c r="F14" s="82" t="n"/>
       <c r="G14" s="83" t="n"/>
       <c r="H14" s="79" t="n"/>
@@ -3321,7 +3949,7 @@
     <col width="17.6640625" customWidth="1" style="39" min="7" max="7"/>
     <col width="15.6640625" customWidth="1" style="39" min="8" max="8"/>
     <col width="14.88671875" customWidth="1" style="39" min="9" max="9"/>
-    <col width="30.33203125" customWidth="1" style="125" min="10" max="10"/>
+    <col width="30.33203125" customWidth="1" style="133" min="10" max="10"/>
     <col width="3.109375" customWidth="1" style="39" min="11" max="11"/>
     <col width="8.88671875" customWidth="1" style="39" min="12" max="16384"/>
   </cols>
@@ -3335,124 +3963,124 @@
       </c>
     </row>
     <row r="2" ht="41.25" customHeight="1" thickBot="1">
-      <c r="B2" s="147" t="inlineStr">
+      <c r="B2" s="154" t="inlineStr">
         <is>
           <t>PFMEA - Occurrence
 The team should agree on the criteria and ranking values. Select one way and consistently apply that scale.</t>
         </is>
       </c>
-      <c r="C2" s="148" t="n"/>
-      <c r="D2" s="148" t="n"/>
-      <c r="E2" s="148" t="n"/>
-      <c r="F2" s="148" t="n"/>
-      <c r="G2" s="148" t="n"/>
-      <c r="H2" s="148" t="n"/>
-      <c r="I2" s="148" t="n"/>
-      <c r="J2" s="149" t="n"/>
+      <c r="C2" s="155" t="n"/>
+      <c r="D2" s="155" t="n"/>
+      <c r="E2" s="155" t="n"/>
+      <c r="F2" s="155" t="n"/>
+      <c r="G2" s="155" t="n"/>
+      <c r="H2" s="155" t="n"/>
+      <c r="I2" s="155" t="n"/>
+      <c r="J2" s="156" t="n"/>
     </row>
     <row r="3" ht="26.25" customHeight="1" thickBot="1">
-      <c r="B3" s="132" t="inlineStr">
+      <c r="B3" s="134" t="inlineStr">
         <is>
           <t>References</t>
         </is>
       </c>
-      <c r="C3" s="132" t="inlineStr">
+      <c r="C3" s="134" t="inlineStr">
         <is>
           <t>J1739</t>
         </is>
       </c>
-      <c r="D3" s="132" t="inlineStr">
+      <c r="D3" s="134" t="inlineStr">
         <is>
           <t>AS13004</t>
         </is>
       </c>
-      <c r="E3" s="148" t="n"/>
-      <c r="F3" s="148" t="n"/>
-      <c r="G3" s="149" t="n"/>
-      <c r="H3" s="132" t="inlineStr">
+      <c r="E3" s="155" t="n"/>
+      <c r="F3" s="155" t="n"/>
+      <c r="G3" s="156" t="n"/>
+      <c r="H3" s="134" t="inlineStr">
         <is>
           <t>AIAG FMEA - 4th Edition</t>
         </is>
       </c>
-      <c r="I3" s="132" t="inlineStr">
+      <c r="I3" s="134" t="inlineStr">
         <is>
           <t>J1739</t>
         </is>
       </c>
-      <c r="J3" s="122" t="inlineStr">
+      <c r="J3" s="124" t="inlineStr">
         <is>
           <t>Examples</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" thickBot="1">
-      <c r="B4" s="122" t="inlineStr">
+      <c r="B4" s="124" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="C4" s="122" t="inlineStr">
+      <c r="C4" s="124" t="inlineStr">
         <is>
           <t>Likelihood of
 Failure</t>
         </is>
       </c>
-      <c r="D4" s="122" t="inlineStr">
+      <c r="D4" s="124" t="inlineStr">
         <is>
           <t>Low volume production</t>
         </is>
       </c>
-      <c r="E4" s="149" t="n"/>
-      <c r="F4" s="122" t="inlineStr">
+      <c r="E4" s="156" t="n"/>
+      <c r="F4" s="124" t="inlineStr">
         <is>
           <t>Process PPM</t>
         </is>
       </c>
-      <c r="G4" s="122" t="inlineStr">
+      <c r="G4" s="124" t="inlineStr">
         <is>
           <t>Time-Based Example</t>
         </is>
       </c>
-      <c r="H4" s="122" t="inlineStr">
+      <c r="H4" s="124" t="inlineStr">
         <is>
           <t>High volume production</t>
         </is>
       </c>
-      <c r="I4" s="149" t="n"/>
-      <c r="J4" s="152" t="n"/>
+      <c r="I4" s="156" t="n"/>
+      <c r="J4" s="159" t="n"/>
     </row>
     <row r="5" ht="29.4" customHeight="1" thickBot="1">
-      <c r="B5" s="150" t="n"/>
-      <c r="C5" s="150" t="n"/>
-      <c r="D5" s="122" t="inlineStr">
+      <c r="B5" s="157" t="n"/>
+      <c r="C5" s="157" t="n"/>
+      <c r="D5" s="124" t="inlineStr">
         <is>
           <t>Likelihood of Cause</t>
         </is>
       </c>
-      <c r="E5" s="122" t="inlineStr">
+      <c r="E5" s="124" t="inlineStr">
         <is>
           <t>Time-Based Example</t>
         </is>
       </c>
-      <c r="F5" s="150" t="n"/>
-      <c r="G5" s="150" t="n"/>
-      <c r="H5" s="122" t="inlineStr">
+      <c r="F5" s="157" t="n"/>
+      <c r="G5" s="157" t="n"/>
+      <c r="H5" s="124" t="inlineStr">
         <is>
           <t>Likelihood of Cause</t>
         </is>
       </c>
-      <c r="I5" s="122" t="inlineStr">
+      <c r="I5" s="124" t="inlineStr">
         <is>
           <t>Incidents per item/unit</t>
         </is>
       </c>
-      <c r="J5" s="150" t="n"/>
+      <c r="J5" s="157" t="n"/>
     </row>
     <row r="6" ht="41.25" customHeight="1" thickBot="1">
       <c r="B6" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="C6" s="123" t="inlineStr">
+      <c r="C6" s="131" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
@@ -3462,7 +4090,7 @@
           <t>100% of production</t>
         </is>
       </c>
-      <c r="E6" s="123" t="inlineStr">
+      <c r="E6" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per occurrence per shift</t>
         </is>
@@ -3470,7 +4098,7 @@
       <c r="F6" s="62" t="n">
         <v>500000</v>
       </c>
-      <c r="G6" s="123" t="inlineStr">
+      <c r="G6" s="131" t="inlineStr">
         <is>
           <t>&gt; 1 per occurrence per shift</t>
         </is>
@@ -3480,7 +4108,7 @@
           <t>1 in 10</t>
         </is>
       </c>
-      <c r="I6" s="123" t="inlineStr">
+      <c r="I6" s="131" t="inlineStr">
         <is>
           <t>&gt; 100 per thousand</t>
         </is>
@@ -3491,7 +4119,7 @@
       <c r="B7" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="C7" s="123" t="inlineStr">
+      <c r="C7" s="131" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3501,7 +4129,7 @@
           <t>50% of production</t>
         </is>
       </c>
-      <c r="E7" s="123" t="inlineStr">
+      <c r="E7" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per occurrence per day</t>
         </is>
@@ -3509,12 +4137,12 @@
       <c r="F7" s="62" t="n">
         <v>50000</v>
       </c>
-      <c r="G7" s="123" t="inlineStr">
+      <c r="G7" s="131" t="inlineStr">
         <is>
           <t>&gt; 1 per occurrence per day</t>
         </is>
       </c>
-      <c r="H7" s="123" t="inlineStr">
+      <c r="H7" s="131" t="inlineStr">
         <is>
           <t>1 in 20</t>
         </is>
@@ -3530,13 +4158,13 @@
       <c r="B8" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="152" t="n"/>
+      <c r="C8" s="159" t="n"/>
       <c r="D8" s="61" t="inlineStr">
         <is>
           <t>20% of production</t>
         </is>
       </c>
-      <c r="E8" s="123" t="inlineStr">
+      <c r="E8" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per 2-3 days</t>
         </is>
@@ -3544,12 +4172,12 @@
       <c r="F8" s="62" t="n">
         <v>20000</v>
       </c>
-      <c r="G8" s="123" t="inlineStr">
+      <c r="G8" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per 2-3 days</t>
         </is>
       </c>
-      <c r="H8" s="123" t="inlineStr">
+      <c r="H8" s="131" t="inlineStr">
         <is>
           <t>1 in 50</t>
         </is>
@@ -3565,13 +4193,13 @@
       <c r="B9" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="150" t="n"/>
+      <c r="C9" s="157" t="n"/>
       <c r="D9" s="61" t="inlineStr">
         <is>
           <t>10% of production</t>
         </is>
       </c>
-      <c r="E9" s="123" t="inlineStr">
+      <c r="E9" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per week</t>
         </is>
@@ -3579,12 +4207,12 @@
       <c r="F9" s="62" t="n">
         <v>10000</v>
       </c>
-      <c r="G9" s="123" t="inlineStr">
+      <c r="G9" s="131" t="inlineStr">
         <is>
           <t>&gt; 1 per week</t>
         </is>
       </c>
-      <c r="H9" s="123" t="inlineStr">
+      <c r="H9" s="131" t="inlineStr">
         <is>
           <t>1 in 100</t>
         </is>
@@ -3600,7 +4228,7 @@
       <c r="B10" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="123" t="inlineStr">
+      <c r="C10" s="131" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
@@ -3610,7 +4238,7 @@
           <t>5% of production</t>
         </is>
       </c>
-      <c r="E10" s="123" t="inlineStr">
+      <c r="E10" s="131" t="inlineStr">
         <is>
           <t>1 per month</t>
         </is>
@@ -3618,12 +4246,12 @@
       <c r="F10" s="62" t="n">
         <v>5000</v>
       </c>
-      <c r="G10" s="123" t="inlineStr">
+      <c r="G10" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per 2 weeks</t>
         </is>
       </c>
-      <c r="H10" s="123" t="inlineStr">
+      <c r="H10" s="131" t="inlineStr">
         <is>
           <t>1 in 500</t>
         </is>
@@ -3639,13 +4267,13 @@
       <c r="B11" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="152" t="n"/>
+      <c r="C11" s="159" t="n"/>
       <c r="D11" s="61" t="inlineStr">
         <is>
           <t>0.5% of production</t>
         </is>
       </c>
-      <c r="E11" s="123" t="inlineStr">
+      <c r="E11" s="131" t="inlineStr">
         <is>
           <t>2 per year</t>
         </is>
@@ -3653,12 +4281,12 @@
       <c r="F11" s="62" t="n">
         <v>1000</v>
       </c>
-      <c r="G11" s="123" t="inlineStr">
+      <c r="G11" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per quarter</t>
         </is>
       </c>
-      <c r="H11" s="123" t="inlineStr">
+      <c r="H11" s="131" t="inlineStr">
         <is>
           <t>1 in 2,000</t>
         </is>
@@ -3674,26 +4302,26 @@
       <c r="B12" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="150" t="n"/>
+      <c r="C12" s="157" t="n"/>
       <c r="D12" s="61" t="inlineStr">
         <is>
           <t>0.1% of production</t>
         </is>
       </c>
-      <c r="E12" s="123" t="inlineStr">
+      <c r="E12" s="131" t="inlineStr">
         <is>
           <t>1 per year</t>
         </is>
       </c>
-      <c r="F12" s="123" t="n">
+      <c r="F12" s="131" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="123" t="inlineStr">
+      <c r="G12" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per half year</t>
         </is>
       </c>
-      <c r="H12" s="123" t="inlineStr">
+      <c r="H12" s="131" t="inlineStr">
         <is>
           <t>1 in 10,000</t>
         </is>
@@ -3709,7 +4337,7 @@
       <c r="B13" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="123" t="inlineStr">
+      <c r="C13" s="131" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3719,20 +4347,20 @@
           <t>0.05% of production</t>
         </is>
       </c>
-      <c r="E13" s="123" t="inlineStr">
+      <c r="E13" s="131" t="inlineStr">
         <is>
           <t>1 per 5 years</t>
         </is>
       </c>
-      <c r="F13" s="123" t="n">
+      <c r="F13" s="131" t="n">
         <v>10</v>
       </c>
-      <c r="G13" s="123" t="inlineStr">
+      <c r="G13" s="131" t="inlineStr">
         <is>
           <t>&gt;1 per year</t>
         </is>
       </c>
-      <c r="H13" s="123" t="inlineStr">
+      <c r="H13" s="131" t="inlineStr">
         <is>
           <t>1 in 100,000</t>
         </is>
@@ -3748,26 +4376,26 @@
       <c r="B14" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="150" t="n"/>
+      <c r="C14" s="157" t="n"/>
       <c r="D14" s="61" t="inlineStr">
         <is>
           <t>0.01% of production</t>
         </is>
       </c>
-      <c r="E14" s="123" t="inlineStr">
+      <c r="E14" s="131" t="inlineStr">
         <is>
           <t>1 per 10 years</t>
         </is>
       </c>
-      <c r="F14" s="123" t="n">
+      <c r="F14" s="131" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="123" t="inlineStr">
+      <c r="G14" s="131" t="inlineStr">
         <is>
           <t>&lt;1 per year</t>
         </is>
       </c>
-      <c r="H14" s="123" t="inlineStr">
+      <c r="H14" s="131" t="inlineStr">
         <is>
           <t>1 in 1,000,000</t>
         </is>
@@ -3783,7 +4411,7 @@
       <c r="B15" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="123" t="inlineStr">
+      <c r="C15" s="131" t="inlineStr">
         <is>
           <t>Very Low</t>
         </is>
@@ -3793,17 +4421,17 @@
           <t>Less than 0.01% of production</t>
         </is>
       </c>
-      <c r="E15" s="123" t="inlineStr">
+      <c r="E15" s="131" t="inlineStr">
         <is>
           <t>&lt;1 per 10 years</t>
         </is>
       </c>
-      <c r="F15" s="123" t="inlineStr">
+      <c r="F15" s="131" t="inlineStr">
         <is>
           <t>zero</t>
         </is>
       </c>
-      <c r="G15" s="123" t="inlineStr">
+      <c r="G15" s="131" t="inlineStr">
         <is>
           <t>Never</t>
         </is>
@@ -3840,7 +4468,7 @@
       </c>
     </row>
     <row r="17" hidden="1">
-      <c r="B17" s="124" t="n"/>
+      <c r="B17" s="132" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="70" t="n"/>
@@ -3856,8 +4484,8 @@
       <c r="B20" s="71" t="n"/>
       <c r="C20" s="71" t="n"/>
       <c r="D20" s="72" t="n"/>
-      <c r="H20" s="125" t="n"/>
-      <c r="I20" s="125" t="n"/>
+      <c r="H20" s="133" t="n"/>
+      <c r="I20" s="133" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="71" t="n"/>
@@ -3878,9 +4506,9 @@
     <mergeCell ref="J3:J5"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="C10:C12"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B2:J2"/>
     <mergeCell ref="C13:C14"/>
-    <mergeCell ref="B2:J2"/>
-    <mergeCell ref="B17:I17"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="H20:I21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" prompt="These columns are not intended to &quot;equal&quot; one another, but serve as a reference that the cross functional team may use to rank process occurrence."/>
@@ -3933,73 +4561,73 @@
       </c>
     </row>
     <row r="2" ht="45.75" customHeight="1" thickBot="1">
-      <c r="B2" s="147" t="inlineStr">
+      <c r="B2" s="154" t="inlineStr">
         <is>
           <t>PFMEA - Severity
 The team should agree on the criteria and ranking values. Select one way and consistently apply that scale.</t>
         </is>
       </c>
-      <c r="C2" s="148" t="n"/>
-      <c r="D2" s="148" t="n"/>
-      <c r="E2" s="148" t="n"/>
-      <c r="F2" s="148" t="n"/>
-      <c r="G2" s="149" t="n"/>
+      <c r="C2" s="155" t="n"/>
+      <c r="D2" s="155" t="n"/>
+      <c r="E2" s="155" t="n"/>
+      <c r="F2" s="155" t="n"/>
+      <c r="G2" s="156" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" thickBot="1">
-      <c r="B3" s="132" t="inlineStr">
+      <c r="B3" s="134" t="inlineStr">
         <is>
           <t>References</t>
         </is>
       </c>
-      <c r="C3" s="132" t="inlineStr">
+      <c r="C3" s="134" t="inlineStr">
         <is>
           <t>Modified from J1739 / AS13004</t>
         </is>
       </c>
-      <c r="D3" s="148" t="n"/>
-      <c r="E3" s="148" t="n"/>
-      <c r="F3" s="149" t="n"/>
-      <c r="G3" s="122" t="inlineStr">
+      <c r="D3" s="155" t="n"/>
+      <c r="E3" s="155" t="n"/>
+      <c r="F3" s="156" t="n"/>
+      <c r="G3" s="124" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
       </c>
     </row>
     <row r="4" ht="29.4" customHeight="1" thickBot="1">
-      <c r="B4" s="122" t="inlineStr">
+      <c r="B4" s="124" t="inlineStr">
         <is>
           <t>Effect</t>
         </is>
       </c>
-      <c r="C4" s="122" t="inlineStr">
+      <c r="C4" s="124" t="inlineStr">
         <is>
           <t>Severity of Effect on Product (Customer Effect)</t>
         </is>
       </c>
-      <c r="D4" s="122" t="inlineStr">
+      <c r="D4" s="124" t="inlineStr">
         <is>
           <t>Ranking</t>
         </is>
       </c>
-      <c r="E4" s="122" t="inlineStr">
+      <c r="E4" s="124" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="F4" s="122" t="inlineStr">
+      <c r="F4" s="124" t="inlineStr">
         <is>
           <t>Severity of Effect on Process (Manufacturing / Assembly Effect)</t>
         </is>
       </c>
-      <c r="G4" s="150" t="n"/>
+      <c r="G4" s="157" t="n"/>
     </row>
     <row r="5" ht="42" customHeight="1" thickBot="1">
-      <c r="B5" s="123" t="inlineStr">
+      <c r="B5" s="131" t="inlineStr">
         <is>
           <t>Failure to meet safety and/or regulatory requirements</t>
         </is>
       </c>
-      <c r="C5" s="123" t="inlineStr">
+      <c r="C5" s="131" t="inlineStr">
         <is>
           <t>Potential failure mode affects safe operation and/or involves noncompliance with regulations without warning</t>
         </is>
@@ -4007,12 +4635,12 @@
       <c r="D5" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="E5" s="123" t="inlineStr">
+      <c r="E5" s="131" t="inlineStr">
         <is>
           <t>Failure to meet safety and/or regulatory requirements</t>
         </is>
       </c>
-      <c r="F5" s="123" t="inlineStr">
+      <c r="F5" s="131" t="inlineStr">
         <is>
           <t>May endanger operator, machine or assembly without warning.</t>
         </is>
@@ -4020,8 +4648,8 @@
       <c r="G5" s="46" t="n"/>
     </row>
     <row r="6" ht="42" customHeight="1" thickBot="1">
-      <c r="B6" s="150" t="n"/>
-      <c r="C6" s="123" t="inlineStr">
+      <c r="B6" s="157" t="n"/>
+      <c r="C6" s="131" t="inlineStr">
         <is>
           <t>Potential failure mode affects safe operation and/or involves noncompliance with regulations with warning</t>
         </is>
@@ -4029,8 +4657,8 @@
       <c r="D6" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="E6" s="150" t="n"/>
-      <c r="F6" s="123" t="inlineStr">
+      <c r="E6" s="157" t="n"/>
+      <c r="F6" s="131" t="inlineStr">
         <is>
           <t>May endanger operator, machine or assembly with warning.</t>
         </is>
@@ -4038,12 +4666,12 @@
       <c r="G6" s="46" t="n"/>
     </row>
     <row r="7" ht="57.6" customHeight="1" thickBot="1">
-      <c r="B7" s="123" t="inlineStr">
+      <c r="B7" s="131" t="inlineStr">
         <is>
           <t>Loss or degradation of primary function</t>
         </is>
       </c>
-      <c r="C7" s="123" t="inlineStr">
+      <c r="C7" s="131" t="inlineStr">
         <is>
           <t>Loss of primary function (product inoperable, does not affect safe operation)</t>
         </is>
@@ -4051,12 +4679,12 @@
       <c r="D7" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="123" t="inlineStr">
+      <c r="E7" s="131" t="inlineStr">
         <is>
           <t>Major disruption</t>
         </is>
       </c>
-      <c r="F7" s="123" t="inlineStr">
+      <c r="F7" s="131" t="inlineStr">
         <is>
           <t>100% of product may have to be scrapped. Line shutdown or stop ship.</t>
         </is>
@@ -4064,8 +4692,8 @@
       <c r="G7" s="46" t="n"/>
     </row>
     <row r="8" ht="42" customHeight="1" thickBot="1">
-      <c r="B8" s="150" t="n"/>
-      <c r="C8" s="123" t="inlineStr">
+      <c r="B8" s="157" t="n"/>
+      <c r="C8" s="131" t="inlineStr">
         <is>
           <t>Degradation of primary function (product operable, but at a reduced level of performance)</t>
         </is>
@@ -4073,12 +4701,12 @@
       <c r="D8" s="49" t="n">
         <v>7</v>
       </c>
-      <c r="E8" s="123" t="inlineStr">
+      <c r="E8" s="131" t="inlineStr">
         <is>
           <t>Significant disruption</t>
         </is>
       </c>
-      <c r="F8" s="123" t="inlineStr">
+      <c r="F8" s="131" t="inlineStr">
         <is>
           <t>A portion of the production run may have to be scrapped. Deviation from primary process; decreased line speed or added manpower).</t>
         </is>
@@ -4086,12 +4714,12 @@
       <c r="G8" s="46" t="n"/>
     </row>
     <row r="9" ht="42" customHeight="1" thickBot="1">
-      <c r="B9" s="123" t="inlineStr">
+      <c r="B9" s="131" t="inlineStr">
         <is>
           <t>Loss or degradation of secondary function</t>
         </is>
       </c>
-      <c r="C9" s="123" t="inlineStr">
+      <c r="C9" s="131" t="inlineStr">
         <is>
           <t xml:space="preserve">Loss of secondary function (product operable but service life greatly reduced, convenience item(s) inoperable, customer dissatisfied) </t>
         </is>
@@ -4099,12 +4727,12 @@
       <c r="D9" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="123" t="inlineStr">
+      <c r="E9" s="131" t="inlineStr">
         <is>
           <t>Moderate disruption</t>
         </is>
       </c>
-      <c r="F9" s="123" t="inlineStr">
+      <c r="F9" s="131" t="inlineStr">
         <is>
           <t>100% of production run may have to be reworked off line and accepted</t>
         </is>
@@ -4112,8 +4740,8 @@
       <c r="G9" s="46" t="n"/>
     </row>
     <row r="10" ht="55.8" customHeight="1" thickBot="1">
-      <c r="B10" s="150" t="n"/>
-      <c r="C10" s="123" t="inlineStr">
+      <c r="B10" s="157" t="n"/>
+      <c r="C10" s="131" t="inlineStr">
         <is>
           <t>Degradation of secondary function (product operable but appearance affected, convenience item(s)  operable at a reduced level, customer dissatisfied.</t>
         </is>
@@ -4121,8 +4749,8 @@
       <c r="D10" s="51" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="150" t="n"/>
-      <c r="F10" s="123" t="inlineStr">
+      <c r="E10" s="157" t="n"/>
+      <c r="F10" s="131" t="inlineStr">
         <is>
           <t xml:space="preserve">A proportion of the production run may have to be reworked off line and acepted </t>
         </is>
@@ -4130,12 +4758,12 @@
       <c r="G10" s="46" t="n"/>
     </row>
     <row r="11" ht="42" customHeight="1" thickBot="1">
-      <c r="B11" s="123" t="inlineStr">
+      <c r="B11" s="131" t="inlineStr">
         <is>
           <t>Annoyance</t>
         </is>
       </c>
-      <c r="C11" s="123" t="inlineStr">
+      <c r="C11" s="131" t="inlineStr">
         <is>
           <t>Appearance, fit and finish type items do not conform, defect noticed by most of the customers (&gt;75%)</t>
         </is>
@@ -4143,12 +4771,12 @@
       <c r="D11" s="52" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="123" t="inlineStr">
+      <c r="E11" s="131" t="inlineStr">
         <is>
           <t>Moderate disruption</t>
         </is>
       </c>
-      <c r="F11" s="123" t="inlineStr">
+      <c r="F11" s="131" t="inlineStr">
         <is>
           <t>100% of production run may have to be reworked in station before it is processed.</t>
         </is>
@@ -4156,8 +4784,8 @@
       <c r="G11" s="46" t="n"/>
     </row>
     <row r="12" ht="42" customHeight="1" thickBot="1">
-      <c r="B12" s="152" t="n"/>
-      <c r="C12" s="123" t="inlineStr">
+      <c r="B12" s="159" t="n"/>
+      <c r="C12" s="131" t="inlineStr">
         <is>
           <t>Appearance, fit and finish type items do not conform, defect noticed by about half of the customers (50%)</t>
         </is>
@@ -4165,8 +4793,8 @@
       <c r="D12" s="53" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="150" t="n"/>
-      <c r="F12" s="123" t="inlineStr">
+      <c r="E12" s="157" t="n"/>
+      <c r="F12" s="131" t="inlineStr">
         <is>
           <t>A proportion of the production run may have to be reworked in station before it is processed.</t>
         </is>
@@ -4174,8 +4802,8 @@
       <c r="G12" s="46" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1" thickBot="1">
-      <c r="B13" s="150" t="n"/>
-      <c r="C13" s="123" t="inlineStr">
+      <c r="B13" s="157" t="n"/>
+      <c r="C13" s="131" t="inlineStr">
         <is>
           <t>Appearance, fit and finish type items do not conform, defect noticed by discriminating customers (&lt;25%)</t>
         </is>
@@ -4183,12 +4811,12 @@
       <c r="D13" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="123" t="inlineStr">
+      <c r="E13" s="131" t="inlineStr">
         <is>
           <t>Minor disruption</t>
         </is>
       </c>
-      <c r="F13" s="123" t="inlineStr">
+      <c r="F13" s="131" t="inlineStr">
         <is>
           <t>Slight inconvenience to process, operation or operator.</t>
         </is>
@@ -4196,12 +4824,12 @@
       <c r="G13" s="46" t="n"/>
     </row>
     <row r="14" ht="18.6" customHeight="1" thickBot="1">
-      <c r="B14" s="123" t="inlineStr">
+      <c r="B14" s="131" t="inlineStr">
         <is>
           <t>No effect</t>
         </is>
       </c>
-      <c r="C14" s="123" t="inlineStr">
+      <c r="C14" s="131" t="inlineStr">
         <is>
           <t>No discernible effect</t>
         </is>
@@ -4209,12 +4837,12 @@
       <c r="D14" s="55" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="123" t="inlineStr">
+      <c r="E14" s="131" t="inlineStr">
         <is>
           <t>No effect</t>
         </is>
       </c>
-      <c r="F14" s="123" t="inlineStr">
+      <c r="F14" s="131" t="inlineStr">
         <is>
           <t>No discernible effect</t>
         </is>
@@ -4295,44 +4923,44 @@
       <c r="B2" s="9" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="153" t="inlineStr">
+      <c r="A3" s="160" t="inlineStr">
         <is>
           <t>1.  All provisions of Product Resources' ISO 9001 QMS apply and are implemented.</t>
         </is>
       </c>
-      <c r="B3" s="154" t="n"/>
+      <c r="B3" s="161" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="153" t="inlineStr">
+      <c r="A4" s="160" t="inlineStr">
         <is>
           <t>2.</t>
         </is>
       </c>
-      <c r="B4" s="154" t="n"/>
+      <c r="B4" s="161" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="153" t="inlineStr">
+      <c r="A5" s="160" t="inlineStr">
         <is>
           <t>3.</t>
         </is>
       </c>
-      <c r="B5" s="154" t="n"/>
+      <c r="B5" s="161" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="153" t="inlineStr">
+      <c r="A6" s="160" t="inlineStr">
         <is>
           <t>4.</t>
         </is>
       </c>
-      <c r="B6" s="154" t="n"/>
+      <c r="B6" s="161" t="n"/>
     </row>
     <row r="7" ht="13.8" customHeight="1" thickBot="1">
-      <c r="A7" s="155" t="inlineStr">
+      <c r="A7" s="162" t="inlineStr">
         <is>
           <t>5.</t>
         </is>
       </c>
-      <c r="B7" s="156" t="n"/>
+      <c r="B7" s="163" t="n"/>
     </row>
     <row r="8" ht="14.4" customHeight="1" thickBot="1" thickTop="1">
       <c r="A8" s="5" t="n"/>

</xml_diff>